<commit_message>
chore: prune resolved open items and local tool ignores
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -13242,7 +13242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -13302,57 +13302,57 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="A4" s="11" t="inlineStr"/>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>权威源从xlsx转仓库内YAML/CSV（可行级diff）；词表归一到单一源</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="inlineStr">
-        <is>
-          <t>已完成（field-source.yaml）</t>
-        </is>
-      </c>
+          <t>── 2026-07-07 导师评审引出的待对齐──</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>v1→v2 逐字段迁移映射（68字段去向，含quality_label/failure_modes/color_change落点）</t>
+          <t>【问俊杰·导师K75点名】§7『观察到的现象』粒度：现7项客观多选 vs 只记『生长/不生长』？可带折中案：一级『生长/未生长』必选＋二级现象细分可选（保失败溯源卖点）</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>不适用（批8整库重建，不迁移v1数据）</t>
+          <t>待对齐(问俊杰)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr"/>
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>── 2026-07-07 导师评审引出的待对齐──</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr"/>
+          <t>【问俊杰】SEM覆盖率：组里习惯的叫法/量化方式/单位？（导师问『SEM占比是什么』，已先改名『SEM覆盖率(视场内材料面积占比,%)』）</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>待对齐(问俊杰)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>【问俊杰·导师K75点名】§7『观察到的现象』粒度：现7项客观多选 vs 只记『生长/不生长』？可带折中案：一级『生长/未生长』必选＋二级现象细分可选（保失败溯源卖点）</t>
+          <t>【问俊杰】堆垛类型实际可判到什么粒度（2H/3R？AA/AB/ABC？扭转角？）→ 决定自由文本还是下拉词表</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -13364,12 +13364,12 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>【问俊杰】SEM覆盖率：组里习惯的叫法/量化方式/单位？（导师问『SEM占比是什么』，已先改名『SEM覆盖率(视场内材料面积占比,%)』）</t>
+          <t>【问俊杰】前驱体『外观描述』词表：组里常用前驱体的形态 + 潮解/变质后的典型外观有哪些</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -13381,170 +13381,85 @@
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>【问俊杰】堆垛类型实际可判到什么粒度（2H/3R？AA/AB/ABC？扭转角？）→ 决定自由文本还是下拉词表</t>
+          <t>【回导师】①SEM占比=SEM视场内材料面积覆盖占比（已改名并给定义）；②必填/选填已加图例行+字体强化，表单UI将用红星标必填</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>待对齐(问俊杰)</t>
+          <t>待回复</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>【问俊杰】前驱体『外观描述』词表：组里常用前驱体的形态 + 潮解/变质后的典型外观有哪些</t>
+          <t>【问俊杰】低压CVD的漏率是否逐炉记录，以及应归入装置校验还是实验过程</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>待对齐(问俊杰)</t>
+          <t>待对齐(本轮不记录漏率)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>【回导师】①SEM占比=SEM视场内材料面积覆盖占比（已改名并给定义）；②必填/选填已加图例行+字体强化，表单UI将用红星标必填</t>
+          <t>【问俊杰】多气体比例的组内标准名称；系统当前由同时间段各气体流量派生</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>待回复</t>
+          <t>待对齐(不另存重复比例)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>表单UI：必填红星/选填弱化等明显标识（导师B93提醒）</t>
+          <t>【问俊杰】掺杂体系“基体/主体/本征材料”的最终角色术语与常见括号化学式示例</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>已实现</t>
+          <t>待对齐(结构已支持)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>【已确认】实验前气体置换统一称“气氛置换”（2026-09-04）</t>
+          <t>【问俊杰】压片等前驱体处理方式的最小参数模板</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>待对齐(不阻塞结构实现)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>【问俊杰】低压CVD的漏率是否逐炉记录，以及应归入装置校验还是实验过程</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>待对齐(本轮不记录漏率)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>【问俊杰】多气体比例的组内标准名称；系统当前由同时间段各气体流量派生</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>待对齐(不另存重复比例)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>【问俊杰】掺杂体系“基体/主体/本征材料”的最终角色术语与常见括号化学式示例</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>待对齐(结构已支持)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>【问俊杰】压片等前驱体处理方式的最小参数模板</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
           <t>待对齐(当前使用具名参数—值—单位)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>已定/已改：一等实体字段表 · 记录单元=炉次+样品 · 掺杂→结构类型+components · 观察现象词表 · 降温参数 · R0条件化(相态判别) · AP/LP校验 · v3.4导师评审回改</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>见『v2→v3变更说明』</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: remove open-items sheet and pending notes from field standard
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -10,7 +10,6 @@
     <sheet name="字段草案" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="一等实体字段表" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="v2→v3变更说明" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="待明确清单" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11182,7 +11181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D96"/>
+  <dimension ref="A1:D95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12134,7 +12133,7 @@
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>表头下加必填级别图例行；必填/条件必填字体加粗着色（导师提醒B93）；表单UI红星标识记入待明确清单</t>
+          <t>表头下加必填级别图例行；必填/条件必填字体加粗着色（导师提醒B93）</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -12144,36 +12143,36 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="11" t="inlineStr">
-        <is>
-          <t>未改</t>
-        </is>
-      </c>
+      <c r="A47" s="11" t="inlineStr"/>
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>§7</t>
-        </is>
-      </c>
-      <c r="C47" s="11" t="inlineStr">
-        <is>
-          <t>『观察到的现象』词表粒度（7项多选 vs 只记生长/不生长）——导师K75点名与俊杰确认后再定，见待明确清单#5</t>
-        </is>
-      </c>
-      <c r="D47" s="11" t="inlineStr">
-        <is>
-          <t>待俊杰对齐</t>
-        </is>
-      </c>
+          <t>── review→v3 回退存档（每条给去向）──</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="inlineStr"/>
+      <c r="D47" s="11" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="inlineStr"/>
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>存档</t>
+        </is>
+      </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>── review→v3 回退存档（每条给去向）──</t>
-        </is>
-      </c>
-      <c r="C48" s="11" t="inlineStr"/>
-      <c r="D48" s="11" t="inlineStr"/>
+          <t>湿度</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>review建议升必填(有DOI)；v3=推荐(6/24未升)。保留推荐，复议是否升R0</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>回退备案</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
@@ -12183,12 +12182,12 @@
       </c>
       <c r="B49" s="11" t="inlineStr">
         <is>
-          <t>湿度</t>
+          <t>装置加热区长/泵型号/MFC配置/PID</t>
         </is>
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>review建议升必填(有DOI)；v3=推荐(6/24未升)。保留推荐，复议是否升R0</t>
+          <t>review §4.1B承诺；v3暂缺。留待『装置』实体字段表（下一轮）</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr">
@@ -12205,12 +12204,12 @@
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>装置加热区长/泵型号/MFC配置/PID</t>
+          <t>炉管履历</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>review §4.1B承诺；v3暂缺。留待『装置』实体字段表（下一轮）</t>
+          <t>review想自动累加；6/24定为手填两数字。保留手填+加重置口径说明（手填有漂移风险）</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -12227,12 +12226,12 @@
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
-          <t>炉管履历</t>
+          <t>时序四元组</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>review想自动累加；6/24定为手填两数字。保留手填+加重置口径说明（手填有漂移风险）</t>
+          <t>review对标NOMAD；v3仅一行导入。落地设计见标准§4时序小节：走FileAsset+通道注册，不进payload</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
@@ -12244,44 +12243,44 @@
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>存档</t>
+          <t>v3.5a</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>时序四元组</t>
+          <t>§1b</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>review对标NOMAD；v3仅一行导入。落地设计见标准§4时序小节：走FileAsset+通道注册，不进payload</t>
+          <t>结构类型由下拉多选纠正为单选判别器；选择值驱动填写提示及组成明细显隐/条件必填</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>回退备案</t>
+          <t>用户走查修复</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="11" t="inlineStr">
         <is>
-          <t>v3.5a</t>
+          <t>v3.6</t>
         </is>
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>§1b</t>
+          <t>全表/实体</t>
         </is>
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>结构类型由下拉多选纠正为单选判别器；选择值驱动填写提示及组成明细显隐/条件必填</t>
+          <t>科学契约加固：结构类型与组成明细纳入R0；补衬底批次引用、具名几何、其他气体名称、sccm参考状态及字段级数值边界</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>用户走查修复</t>
+          <t>全库审查修复</t>
         </is>
       </c>
     </row>
@@ -12293,12 +12292,12 @@
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>全表/实体</t>
+          <t>§6–§7</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>科学契约加固：结构类型与组成明细纳入R0；补衬底批次引用、具名几何、其他气体名称、sccm参考状态及字段级数值边界</t>
+          <t>过程事件改为带UTC offset的绝对日期时间；实测层数、覆盖率、畴尺寸、成核密度拆为独立量，关键谱学指标改为带单位的结构化数组</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -12310,22 +12309,22 @@
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
         <is>
-          <t>v3.6</t>
+          <t>v3.7</t>
         </is>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>§6–§7</t>
+          <t>§1–§4</t>
         </is>
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>过程事件改为带UTC offset的绝对日期时间；实测层数、覆盖率、畴尺寸、成核密度拆为独立量，关键谱学指标改为带单位的结构化数组</t>
+          <t>按2026-07-24导师走查：温湿度与预检、目标形态升必填；删除粒子占位；批次引用升必填；前驱体与衬底处理改具名有序数组；衬底晶向、粗糙度、尺寸与倾角结构化</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>全库审查修复</t>
+          <t>导师走查整改</t>
         </is>
       </c>
     </row>
@@ -12337,12 +12336,12 @@
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>§1–§4</t>
+          <t>§5–§6</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>按2026-07-24导师走查：温湿度与预检、目标形态升必填；删除粒子占位；批次引用升必填；前驱体与衬底处理改具名有序数组；衬底晶向、粗糙度、尺寸与倾角结构化</t>
+          <t>11阶段收敛为预处理、反应条件、具名其他记录；温度程序、实测文件、多气体时序、时长、降温、实际外场与事件附件全部改为可校验结构</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -12359,12 +12358,12 @@
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>§5–§6</t>
+          <t>实体</t>
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>11阶段收敛为预处理、反应条件、具名其他记录；温度程序、实测文件、多气体时序、时长、降温、实际外场与事件附件全部改为可校验结构</t>
+          <t>Setup删除sccm参考值、加热区长度、泵、MFC和PID，坐标系固定，新增温度传感器；炉管材质与形状拆入具名对象；MaterialLot新增瓶身或包装标签附件</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
@@ -12376,22 +12375,22 @@
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>v3.7</t>
+          <t>v3.8</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>实体</t>
+          <t>§1–§5</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Setup删除sccm参考值、加热区长度、泵、MFC和PID，坐标系固定，新增温度传感器；炉管材质与形状拆入具名对象；MaterialLot新增瓶身或包装标签附件</t>
+          <t>用户走查修复：炉管和各舟履历改为每炉手填；炉管尺寸按圆/方/矩形条件展开；前驱体源温改为可选位置温度及依据；外场按等离子体/光/电展开明确参数</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>导师走查整改</t>
+          <t>用户走查修复</t>
         </is>
       </c>
     </row>
@@ -12403,12 +12402,12 @@
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
-          <t>§1–§5</t>
+          <t>§4/实体</t>
         </is>
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>用户走查修复：炉管和各舟履历改为每炉手填；炉管尺寸按圆/方/矩形条件展开；前驱体源温改为可选位置温度及依据；外场按等离子体/光/电展开明确参数</t>
+          <t>衬底稳定规格归MaterialLot：晶向抛光、偏切角与方向、氧化层及标称粗糙度由批次冻结带出；本片尺寸、放置、预处理和位置留在炉次；气瓶等级改为供应商原始标签选填</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
@@ -12425,12 +12424,12 @@
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>§4/实体</t>
+          <t>术语/表征</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>衬底稳定规格归MaterialLot：晶向抛光、偏切角与方向、氧化层及标称粗糙度由批次冻结带出；本片尺寸、放置、预处理和位置留在炉次；气瓶等级改为供应商原始标签选填</t>
+          <t>装置与实际外场统一显示“等离子体”；体相空间群改用内置230项检索；“表征方法”与仪器引用分开，固定配置只记录稳定硬件能力</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
@@ -12442,127 +12441,127 @@
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
         <is>
-          <t>v3.8</t>
+          <t>v3.9</t>
         </is>
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>术语/表征</t>
+          <t>§1/§4/实体</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>装置与实际外场统一显示“等离子体”；体相空间群改用内置230项检索；“表征方法”与仪器引用分开，固定配置只记录稳定硬件能力</t>
+          <t>按会议逐字稿删除悬浮粒子浓度；粗糙度允许明确记录供应商未提供；旧批次缺稳定字段时禁止在实验回填；区分来料尺寸与本次实际切片尺寸</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>用户走查修复</t>
+          <t>2026-07-25用户复核</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>v3.9</t>
+          <t>v3.10</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>§1/§4/实体</t>
+          <t>§3/§4/实体</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>按会议逐字稿删除悬浮粒子浓度；粗糙度允许明确记录供应商未提供；旧批次缺稳定字段时禁止在实验回填；区分来料尺寸与本次实际切片尺寸</t>
+          <t>补齐温区距离参照、条件不适用后端约束与旧等离子别名；粒径/形态按物料类别展开；晶向抛光和偏切以有规格、未提供、不适用三态记录，禁止用伪值或0代替未知</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>2026-07-25用户复核</t>
+          <t>2026-07-25终审收口</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="inlineStr">
         <is>
-          <t>v3.10</t>
+          <t>v3.11</t>
         </is>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>§3/§4/实体</t>
+          <t>§6/实体</t>
         </is>
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>补齐温区距离参照、条件不适用后端约束与旧等离子别名；粒径/形态按物料类别展开；晶向抛光和偏切以有规格、未提供、不适用三态记录，禁止用伪值或0代替未知</t>
+          <t>事件具体说明始终可选填写、终止原因=其他时升级为必填；仪器字段改称“适用表征方法”；补明热电偶距离与前驱体温区、炉管截面与尺寸的联动必填规则</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr">
         <is>
-          <t>2026-07-25终审收口</t>
+          <t>2026-07-25逐字稿与语义终审</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>v3.11</t>
+          <t>v3.12</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
-          <t>§6/实体</t>
+          <t>§1–§5/实体</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>事件具体说明始终可选填写、终止原因=其他时升级为必填；仪器字段改称“适用表征方法”；补明热电偶距离与前驱体温区、炉管截面与尺寸的联动必填规则</t>
+          <t>制备终版整改：新记录固定CVD顶层方法；目标产物按掺杂、合金、材料层和区域填写；Setup逐温区只填传感器类型与温度测量误差；前驱体角色与样片标记必填；压力类别和值成对；反应删除伪循环派生</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>2026-07-25逐字稿与语义终审</t>
+          <t>2026-07-27终版整改</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
         <is>
-          <t>v3.12</t>
+          <t>v3.13</t>
         </is>
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
-          <t>§1–§5/实体</t>
+          <t>§1b</t>
         </is>
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>制备终版整改：新记录固定CVD顶层方法；目标产物按掺杂、合金、材料层和区域填写；Setup逐温区只填传感器类型与温度测量误差；前驱体角色与样片标记必填；压力类别和值成对；反应删除伪循环派生</t>
+          <t>目标产物复核：化学式示例按结构类型变化；删除“普通数字”用户文案；掺杂区只显示掺杂元素；空间群按化学式给出经核对的常见体相候选并保留230项搜索；异质结构逐层或逐区域填写空间群</t>
         </is>
       </c>
       <c r="D65" s="11" t="inlineStr">
         <is>
-          <t>2026-07-27终版整改</t>
+          <t>2026-07-28用户逐项复核</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>v3.13</t>
+          <t>v3.15</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>§1b</t>
+          <t>实体/设备</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>目标产物复核：化学式示例按结构类型变化；删除“普通数字”用户文案；掺杂区只显示掺杂元素；空间群按化学式给出经核对的常见体相候选并保留230项搜索；异质结构逐层或逐区域填写空间群</t>
+          <t>温度传感器由热电偶分型号改为按测温原理选择类别：热电偶、热电阻（RTD）、红外测温仪、光纤温度传感器、热敏电阻、其他</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr">
@@ -12574,7 +12573,7 @@
     <row r="67">
       <c r="A67" s="11" t="inlineStr">
         <is>
-          <t>v3.15</t>
+          <t>v3.16</t>
         </is>
       </c>
       <c r="B67" s="11" t="inlineStr">
@@ -12584,7 +12583,7 @@
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>温度传感器由热电偶分型号改为按测温原理选择类别：热电偶、热电阻（RTD）、红外测温仪、光纤温度传感器、热敏电阻、其他</t>
+          <t>Setup拆分制造商或品牌与型号，增加装置来源；实验室装置编号保持唯一但允许管理员通过新版本纠错；温区标称测温精度改为选填</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr">
@@ -12596,7 +12595,7 @@
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>v3.16</t>
+          <t>v3.17</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
@@ -12606,7 +12605,7 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>Setup拆分制造商或品牌与型号，增加装置来源；实验室装置编号保持唯一但允许管理员通过新版本纠错；温区标称测温精度改为选填</t>
+          <t>装置来源改为必填；商业设备显示制造商与型号，实验室自制显示设计或建造单位与内部型号，改造设备显示原设备制造商、原设备型号与改造内容；公共技术字段不变</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr">
@@ -12618,105 +12617,105 @@
     <row r="69">
       <c r="A69" s="11" t="inlineStr">
         <is>
-          <t>v3.17</t>
+          <t>v3.18</t>
         </is>
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>实体/设备</t>
+          <t>§3/实体</t>
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>装置来源改为必填；商业设备显示制造商与型号，实验室自制显示设计或建造单位与内部型号，改造设备显示原设备制造商、原设备型号与改造内容；公共技术字段不变</t>
+          <t>前驱体先选本次使用形态再筛选批次；删除炉次中重复的名称化学式和CAS；用途、使用量、使用前状态、处理步骤按实际语义收敛；非气态按舟、坩埚、衬底表面或其他容器展开容器尺寸、履历与炉内位置</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28用户逐项复核</t>
+          <t>2026-07-28前驱体首版复核</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>v3.18</t>
+          <t>v4.0-rc.1</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>§3/实体</t>
+          <t>科学对象/实体/结果</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>前驱体先选本次使用形态再筛选批次；删除炉次中重复的名称化学式和CAS；用途、使用量、使用前状态、处理步骤按实际语义收敛；非气态按舟、坩埚、衬底表面或其他容器展开容器尺寸、履历与炉内位置</t>
+          <t>引入正交TargetSpec、物理SourceLoad、统一ProcessTimeline、不可变RunRevision、样品转换图及MeasurementRun→AnalysisRun→PropertyValue/MaterialAssertion溯源链；物料、装置部件和仪器能力补齐归一化字段；PVD不进入发布契约</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28前驱体首版复核</t>
+          <t>2026-07-28深度审查整改</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="11" t="inlineStr">
         <is>
-          <t>v4.0-rc.1</t>
+          <t>v4.0-alpha.2</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>科学对象/实体/结果</t>
+          <t>科学完整性复核</t>
         </is>
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>引入正交TargetSpec、物理SourceLoad、统一ProcessTimeline、不可变RunRevision、样品转换图及MeasurementRun→AnalysisRun→PropertyValue/MaterialAssertion溯源链；物料、装置部件和仪器能力补齐归一化字段；PVD不进入发布契约</t>
+          <t>关闭旧结果写入与手工派生入口；收紧审阅和转化权限；修正跨炉次转化溯源、过程单位归一化、不可变修订导出及数据集查询语义；冻结装料容器、测量时校准和样品—修订关联快照；状态降为内部验证</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr">
         <is>
-          <t>2026-07-28深度审查整改</t>
+          <t>2026-07-29二次复核整改</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.2</t>
+          <t>v4.0-alpha.3</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>科学完整性复核</t>
+          <t>§4 衬底</t>
         </is>
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>关闭旧结果写入与手工派生入口；收紧审阅和转化权限；修正跨炉次转化溯源、过程单位归一化、不可变修订导出及数据集查询语义；冻结装料容器、测量时校准和样品—修订关联快照；状态降为内部验证</t>
+          <t>产品简化界面增加本片轴向位置与备注；轴向位置为普通用户提交前必填，不暴露三维坐标</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>2026-07-29二次复核整改</t>
+          <t>2026-07-30产品简化</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.3</t>
+          <t>v4.0-alpha.4</t>
         </is>
       </c>
       <c r="B73" s="11" t="inlineStr">
         <is>
-          <t>§4 衬底</t>
+          <t>§7 表征</t>
         </is>
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>产品简化界面增加本片轴向位置与备注；轴向位置为普通用户提交前必填，不暴露三维坐标</t>
+          <t>表征方法拆分最小必填与更多测量参数，固定各方法常用结果项，并增加“其他”方法说明；科学对象仍由后端统一落库</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr">
@@ -12728,29 +12727,29 @@
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.4</t>
+          <t>v4.0-alpha.5</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>§7 表征</t>
+          <t>实体/物料批次</t>
         </is>
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>表征方法拆分最小必填与更多测量参数，固定各方法常用结果项，并增加“其他”方法说明；科学对象仍由后端统一落库</t>
+          <t>CAS号与数值纯度改为有来源才选填；删除同义名、标识符、商业规格JSON、纯度基准/来源及D50四字段；供应商规格或等级按标签原文照录</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>2026-07-30产品简化</t>
+          <t>2026-08-02供应商资料复核与减负</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.5</t>
+          <t>v4.0-alpha.6</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
@@ -12760,19 +12759,19 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>CAS号与数值纯度改为有来源才选填；删除同义名、标识符、商业规格JSON、纯度基准/来源及D50四字段；供应商规格或等级按标签原文照录</t>
+          <t>物料表单文案正式化：常规字段说明改为简短占位示例，仅为纯度及衬底规格等易误录字段保留必要说明；统一字段名称、中文标点和中英文术语</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr">
         <is>
-          <t>2026-08-02供应商资料复核与减负</t>
+          <t>2026-08-02用户界面复核</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.6</t>
+          <t>v4.0-alpha.7</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
@@ -12782,19 +12781,19 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>物料表单文案正式化：常规字段说明改为简短占位示例，仅为纯度及衬底规格等易误录字段保留必要说明；统一字段名称、中文标点和中英文术语</t>
+          <t>化学式复用目标产物输入控件并提示元素与语法；货号与批号直接对应包装上的 Cat./Product No. 和 Lot/Batch No.，说明两者的产品与实物批次分工</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>2026-08-02用户界面复核</t>
+          <t>2026-08-06用户界面复核</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.7</t>
+          <t>v4.0-alpha.8</t>
         </is>
       </c>
       <c r="B77" s="11" t="inlineStr">
@@ -12804,7 +12803,7 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>化学式复用目标产物输入控件并提示元素与语法；货号与批号直接对应包装上的 Cat./Product No. 和 Lot/Batch No.，说明两者的产品与实物批次分工</t>
+          <t>删除化学式格式说明，只保留示例与即时元素/语法反馈</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr">
@@ -12816,7 +12815,7 @@
     <row r="78">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.8</t>
+          <t>v4.0-alpha.9</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
@@ -12826,7 +12825,7 @@
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>删除化学式格式说明，只保留示例与即时元素/语法反馈</t>
+          <t>供应商“其他”改为明确的新增供应商与名称输入；供应商规格或等级改为产品等级（标签原文），说明资料未标注时留空</t>
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr">
@@ -12838,17 +12837,17 @@
     <row r="79">
       <c r="A79" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.9</t>
+          <t>v4.0-alpha.12</t>
         </is>
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>实体/物料批次</t>
+          <t>§5 生长条件</t>
         </is>
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>供应商“其他”改为明确的新增供应商与名称输入；供应商规格或等级改为产品等级（标签原文），说明资料未标注时留空</t>
+          <t>统一实验时间零点与有效生长窗口；补齐气体批次、流量来源、绝对压力、受控降温速率、实际外场参数和多条异常事件，并自动覆盖生长后的实验过程</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr">
@@ -12860,7 +12859,7 @@
     <row r="80">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.12</t>
+          <t>v4.0-alpha.13</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
@@ -12870,19 +12869,19 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>统一实验时间零点与有效生长窗口；补齐气体批次、流量来源、绝对压力、受控降温速率、实际外场参数和多条异常事件，并自动覆盖生长后的实验过程</t>
+          <t>将容易误解为管理制度的“压力制度/压力体系”统一改为“反应压力条件”，数据字段与校验规则不变</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>2026-08-06用户界面复核</t>
+          <t>2026-08-07用户界面复核</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.13</t>
+          <t>v4.0-alpha.14</t>
         </is>
       </c>
       <c r="B81" s="11" t="inlineStr">
@@ -12892,7 +12891,7 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>将容易误解为管理制度的“压力制度/压力体系”统一改为“反应压力条件”，数据字段与校验规则不变</t>
+          <t>改为按实际操作和持续时间录入，系统自动生成系统准备、升温与预处理、反应、反应后处理和降温时间轴；气体优先选择使用阶段，仅自定义时填写起止时间</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
@@ -12904,7 +12903,7 @@
     <row r="82">
       <c r="A82" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.14</t>
+          <t>v4.0-alpha.15</t>
         </is>
       </c>
       <c r="B82" s="11" t="inlineStr">
@@ -12914,51 +12913,51 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>改为按实际操作和持续时间录入，系统自动生成系统准备、升温与预处理、反应、反应后处理和降温时间轴；气体优先选择使用阶段，仅自定义时填写起止时间</t>
+          <t>删除缺乏统一文献定义且无法直接观测的反应计时起点、反应开始前用时、反应时长及重复的反应后处理；实际过程由温度步骤、气体时段、系统准备、压力与降温记录</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>2026-08-07用户界面复核</t>
+          <t>2026-08-07用户界面复核与原始论文核对</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.15</t>
+          <t>v4.0-alpha.16</t>
         </is>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>§5 生长条件</t>
+          <t>§3 前驱体装载</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>删除缺乏统一文献定义且无法直接观测的反应计时起点、反应开始前用时、反应时长及重复的反应后处理；实际过程由温度步骤、气体时段、系统准备、压力与降温记录</t>
+          <t>删除偏TMDC的必填单选作用，改为选填多选工艺作用；一次旋涂支持多段转速；衬底表面装载关联稳定衬底片；旋涂物料可成对记录溶液浓度与受控单位</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr">
         <is>
-          <t>2026-08-07用户界面复核与原始论文核对</t>
+          <t>2026-08-12师兄真实试填反馈</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.16</t>
+          <t>v4.0-alpha.17</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>§3 前驱体装载</t>
+          <t>§5 生长条件</t>
         </is>
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>删除偏TMDC的必填单选作用，改为选填多选工艺作用；一次旋涂支持多段转速；衬底表面装载关联稳定衬底片；旋涂物料可成对记录溶液浓度与受控单位</t>
+          <t>气体词表增加二氧化碳，启动混合气与置换气源契约收口</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr">
@@ -12970,496 +12969,242 @@
     <row r="85">
       <c r="A85" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.17</t>
+          <t>v4.0-alpha.18</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>§5 生长条件</t>
+          <t>§1–§6科学修订契约·MaterialLot气瓶</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>气体词表增加二氧化碳，启动混合气与置换气源契约收口</t>
+          <t>气瓶版本结构化登记纯气或预混组成；置换引用实际气瓶版本；基本信息、目标材料、前驱体、过程事件与生长条件的发布字段改用当前不可变修订payload真实key和schema_path，旧扁平字段仅历史兼容</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
         <is>
-          <t>2026-08-12师兄真实试填反馈</t>
+          <t>2026-08-13全链路契约复核</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.18</t>
+          <t>v4.0-alpha.19</t>
         </is>
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>§1–§6科学修订契约·MaterialLot气瓶</t>
+          <t>表征科学属性</t>
         </is>
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>气瓶版本结构化登记纯气或预混组成；置换引用实际气瓶版本；基本信息、目标材料、前驱体、过程事件与生长条件的发布字段改用当前不可变修订payload真实key和schema_path，旧扁平字段仅历史兼容</t>
+          <t>PropertyValue 补齐数值/文本表示类型与物理范围，并统一后端和前端的单一源校验</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr">
         <is>
-          <t>2026-08-13全链路契约复核</t>
+          <t>2026-08-31表征全链路独立审查</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.19</t>
+          <t>v4.0-alpha.20</t>
         </is>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>表征科学属性</t>
+          <t>实体/物料批次</t>
         </is>
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>PropertyValue 补齐数值/文本表示类型与物理范围，并统一后端和前端的单一源校验</t>
+          <t>云母衬底增加白云母、金云母和氟金云母类型选择，并由系统生成理想化学式，避免选择材料后在表单顶部突然出现手填化学式</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr">
         <is>
-          <t>2026-08-31表征全链路独立审查</t>
+          <t>2026-09-01用户试填反馈</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.20</t>
+          <t>v4.0-alpha.21</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>实体/物料批次</t>
+          <t>实体/制备/样品与表征流程</t>
         </is>
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>云母衬底增加白云母、金云母和氟金云母类型选择，并由系统生成理想化学式，避免选择材料后在表单顶部突然出现手填化学式</t>
+          <t>仪器能力改为勾选、日期改为日期控件、装置使用身份标签、异常改为显式确认、表征入口保留样品上下文，并在编辑后清除旧校验错误</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>2026-09-01用户试填反馈</t>
+          <t>2026-09-01全表单交互复核</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.21</t>
+          <t>v4.0-alpha.22</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>实体/制备/样品与表征流程</t>
+          <t>§3/§5 生长条件与装置履历</t>
         </is>
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>仪器能力改为勾选、日期改为日期控件、装置使用身份标签、异常改为显式确认、表征入口保留样品上下文，并在编辑后清除旧校验错误</t>
+          <t>生长条件按实验前准备、温度、气体、反应压力、降温和异常分区；温度步骤移除待判断与初始温度伪时长；异常改为勾选框，并缩短温区和炉管履历文案</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr">
         <is>
-          <t>2026-09-01全表单交互复核</t>
+          <t>2026-09-02用户界面复核</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.22</t>
+          <t>v4.0-alpha.23</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>§3/§5 生长条件与装置履历</t>
+          <t>§1b/§3/§4/§5 制备记录填写体验</t>
         </is>
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>生长条件按实验前准备、温度、气体、反应压力、降温和异常分区；温度步骤移除待判断与初始温度伪时长；异常改为勾选框，并缩短温区和炉管履历文案</t>
+          <t>缩短晶体结构、实验目标、相对测温点位置、使用前处理、衬底处理和压力条件文案；明确必填空状态与提交检查，并减少气体首段录入步骤</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>2026-09-02用户界面复核</t>
+          <t>2026-09-02用户全流程复核</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.23</t>
+          <t>v4.0-alpha.24</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>§1b/§3/§4/§5 制备记录填写体验</t>
+          <t>§5 实验前准备</t>
         </is>
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>缩短晶体结构、实验目标、相对测温点位置、使用前处理、衬底处理和压力条件文案；明确必填空状态与提交检查，并减少气体首段录入步骤</t>
+          <t>抽真空优先记录终点绝对压力；有压力读数时持续时间改为选填，无压力读数时持续时间必填</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr">
         <is>
-          <t>2026-09-02用户全流程复核</t>
+          <t>2026-09-02用户实验前准备复核</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.24</t>
+          <t>v4.0-alpha.26</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>§5 实验前准备</t>
+          <t>§1b 目标材料</t>
         </is>
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>抽真空优先记录终点绝对压力；有压力读数时持续时间改为选填，无压力读数时持续时间必填</t>
+          <t>单一材料改为本征材料，原子层数改为材料层数；删除无法预知的目标覆盖状态和语义混淆的目标生长取向，以目标产物形态和条件平面轮廓表达预期形态</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>2026-09-02用户实验前准备复核</t>
+          <t>2026-09-03用户目标材料复核</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.26</t>
+          <t>v4.0-alpha.27</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>§1b 目标材料</t>
+          <t>装置与衬底</t>
         </is>
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>单一材料改为本征材料，原子层数改为材料层数；删除无法预知的目标覆盖状态和语义混淆的目标生长取向，以目标产物形态和条件平面轮廓表达预期形态</t>
+          <t>外场能力增加具名其他；衬底批号改为按标签提供情况条件填写并补生产日期；衬底处理合并为可展开溶剂清洗，并以紫外/臭氧处理替代笼统亲水处理</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr">
         <is>
-          <t>2026-09-03用户目标材料复核</t>
+          <t>2026-09-03用户装置与衬底复核</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.27</t>
+          <t>v4.0-alpha.35</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>装置与衬底</t>
+          <t>表征客观测量</t>
         </is>
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>外场能力增加具名其他；衬底批号改为按标签提供情况条件填写并补生产日期；衬底处理合并为可展开溶剂清洗，并以紫外/臭氧处理替代笼统亲水处理</t>
+          <t>新表征不分区域、不录入材料判定；谱峰按编号记录峰位、半高全宽和强度，区分未分析与未检出；AFM、电子显微镜、元素定量按方法与模式显示，历史判定不再自动汇总成整片样品结论</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>2026-09-03用户装置与衬底复核</t>
+          <t>2026-09-04用户表征复核</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="11" t="inlineStr">
         <is>
-          <t>v4.0-alpha.35</t>
+          <t>R0</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>表征客观测量</t>
+          <t>最小可复现核心(27项，含条件必填)</t>
         </is>
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>新表征不分区域、不录入材料判定；谱峰按编号记录峰位、半高全宽和强度，区分未分析与未检出；AFM、电子显微镜、元素定量按方法与模式显示，历史判定不再自动汇总成整片样品结论</t>
+          <t>过程R0以温度/气体/压力通道和降温条件为准；不再要求人工划分反应阶段或反应时长</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr">
         <is>
-          <t>2026-09-04用户表征复核</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="11" t="inlineStr">
-        <is>
-          <t>R0</t>
-        </is>
-      </c>
-      <c r="B96" s="11" t="inlineStr">
-        <is>
-          <t>最小可复现核心(27项，含条件必填)</t>
-        </is>
-      </c>
-      <c r="C96" s="11" t="inlineStr">
-        <is>
-          <t>过程R0以温度/气体/压力通道和降温条件为准；不再要求人工划分反应阶段或反应时长</t>
-        </is>
-      </c>
-      <c r="D96" s="11" t="inlineStr">
-        <is>
           <t>必填集</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="64" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>问题</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>状态</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B2" s="11" t="inlineStr">
-        <is>
-          <t>化学式 / 异质结 标准写法（渲染规则，找国标或组内定）</t>
-        </is>
-      </c>
-      <c r="C2" s="11" t="inlineStr">
-        <is>
-          <t>待办</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B3" s="11" t="inlineStr">
-        <is>
-          <t>化学式录入：文本+元素校验/自动补全（建议，非周期表点选）</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="inlineStr">
-        <is>
-          <t>待办(技术)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr"/>
-      <c r="B4" s="11" t="inlineStr">
-        <is>
-          <t>── 2026-07-07 导师评审引出的待对齐──</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>【问俊杰·导师K75点名】§7『观察到的现象』粒度：现7项客观多选 vs 只记『生长/不生长』？可带折中案：一级『生长/未生长』必选＋二级现象细分可选（保失败溯源卖点）</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>待对齐(问俊杰)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>【问俊杰】SEM覆盖率：组里习惯的叫法/量化方式/单位？（导师问『SEM占比是什么』，已先改名『SEM覆盖率(视场内材料面积占比,%)』）</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>待对齐(问俊杰)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>【问俊杰】堆垛类型实际可判到什么粒度（2H/3R？AA/AB/ABC？扭转角？）→ 决定自由文本还是下拉词表</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>待对齐(问俊杰)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>【问俊杰】前驱体『外观描述』词表：组里常用前驱体的形态 + 潮解/变质后的典型外观有哪些</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>待对齐(问俊杰)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>【回导师】①SEM占比=SEM视场内材料面积覆盖占比（已改名并给定义）；②必填/选填已加图例行+字体强化，表单UI将用红星标必填</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>待回复</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>【问俊杰】低压CVD的漏率是否逐炉记录，以及应归入装置校验还是实验过程</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>待对齐(本轮不记录漏率)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>【问俊杰】多气体比例的组内标准名称；系统当前由同时间段各气体流量派生</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>待对齐(不另存重复比例)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>【问俊杰】掺杂体系“基体/主体/本征材料”的最终角色术语与常见括号化学式示例</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>待对齐(结构已支持)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>【问俊杰】压片等前驱体处理方式的最小参数模板</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>待对齐(当前使用具名参数—值—单位)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: remove legacy result model and characterization compatibility layer
</commit_message>
<xml_diff>
--- a/docs/standard/字段草案-v3.xlsx
+++ b/docs/standard/字段草案-v3.xlsx
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K136"/>
+  <dimension ref="A1:K125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6574,7 +6574,7 @@
     <row r="119" ht="20" customHeight="1">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>§7 旧扁平结果字段（未发布；由 MeasurementRun → AnalysisRun → PropertyValue / MaterialAssertion 替代）</t>
+          <t>§8 PVD 专用（若合成方法选 PVD 类才启用；延后实现，先占位）</t>
         </is>
       </c>
       <c r="B119" s="8" t="n"/>
@@ -6591,27 +6591,27 @@
     <row r="120">
       <c r="A120" s="11" t="inlineStr">
         <is>
-          <t>表征</t>
+          <t>PVD</t>
         </is>
       </c>
       <c r="B120" s="11" t="inlineStr">
         <is>
-          <t>表征方法</t>
+          <t>靶材（批次）</t>
         </is>
       </c>
       <c r="C120" s="11" t="inlineStr">
         <is>
-          <t>本次使用的表征手段；仪器通过独立仪器引用选择</t>
+          <t>靶材化学身份 + 批次</t>
         </is>
       </c>
       <c r="D120" s="11" t="inlineStr">
         <is>
-          <t>下拉+其他</t>
+          <t>引用</t>
         </is>
       </c>
       <c r="E120" s="11" t="inlineStr">
         <is>
-          <t>OM/Raman/PL/SHG/AFM/SEM/TEM/XRD/其他/低波数Raman</t>
+          <t>批次库</t>
         </is>
       </c>
       <c r="F120" s="11" t="inlineStr">
@@ -6626,40 +6626,36 @@
       </c>
       <c r="H120" s="11" t="inlineStr">
         <is>
-          <t>Raman</t>
+          <t>MoS₂ 靶-T01</t>
         </is>
       </c>
       <c r="I120" s="11" t="inlineStr">
         <is>
-          <t>会议</t>
-        </is>
-      </c>
-      <c r="J120" s="15" t="inlineStr">
-        <is>
-          <t>★v3：长一批表征一批，拆成独立表编号关联；不要在此字段重复写仪器</t>
-        </is>
-      </c>
+          <t>复审</t>
+        </is>
+      </c>
+      <c r="J120" s="11" t="inlineStr"/>
       <c r="K120" s="11" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="11" t="inlineStr">
         <is>
-          <t>表征</t>
+          <t>PVD</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
         <is>
-          <t>测试条件</t>
+          <t>靶基距</t>
         </is>
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>该表征的测试参数</t>
+          <t>靶到衬底距离</t>
         </is>
       </c>
       <c r="D121" s="11" t="inlineStr">
         <is>
-          <t>文本/自由</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E121" s="11" t="inlineStr">
@@ -6669,7 +6665,7 @@
       </c>
       <c r="F121" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="G121" s="13" t="inlineStr">
@@ -6679,50 +6675,50 @@
       </c>
       <c r="H121" s="11" t="inlineStr">
         <is>
-          <t>激光532 nm；功率1 mW；物镜100×</t>
+          <t>80</t>
         </is>
       </c>
       <c r="I121" s="11" t="inlineStr">
         <is>
-          <t>会议</t>
-        </is>
-      </c>
-      <c r="J121" s="11" t="inlineStr">
-        <is>
-          <t>随仪器导出</t>
-        </is>
-      </c>
-      <c r="K121" s="11" t="inlineStr"/>
+          <t>复审</t>
+        </is>
+      </c>
+      <c r="J121" s="11" t="inlineStr"/>
+      <c r="K121" s="11" t="inlineStr">
+        <is>
+          <t>{"gt":0}</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="11" t="inlineStr">
         <is>
-          <t>表征</t>
+          <t>PVD</t>
         </is>
       </c>
       <c r="B122" s="11" t="inlineStr">
         <is>
-          <t>原始数据</t>
+          <t>功率与偏压</t>
         </is>
       </c>
       <c r="C122" s="11" t="inlineStr">
         <is>
-          <t>上传原始文件（留校验和）</t>
+          <t>DC/RF 功率、基底偏压</t>
         </is>
       </c>
       <c r="D122" s="11" t="inlineStr">
         <is>
-          <t>附件</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E122" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DC/RF</t>
         </is>
       </c>
       <c r="F122" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>W·V</t>
         </is>
       </c>
       <c r="G122" s="13" t="inlineStr">
@@ -6732,12 +6728,12 @@
       </c>
       <c r="H122" s="11" t="inlineStr">
         <is>
-          <t>raman.txt</t>
+          <t>RF 150W；偏压 -50V</t>
         </is>
       </c>
       <c r="I122" s="11" t="inlineStr">
         <is>
-          <t>会议/复审</t>
+          <t>复审</t>
         </is>
       </c>
       <c r="J122" s="11" t="inlineStr"/>
@@ -6746,32 +6742,32 @@
     <row r="123">
       <c r="A123" s="11" t="inlineStr">
         <is>
-          <t>实测产物</t>
+          <t>PVD</t>
         </is>
       </c>
       <c r="B123" s="11" t="inlineStr">
         <is>
-          <t>观察到的现象</t>
+          <t>等离子体气氛与工作气压</t>
         </is>
       </c>
       <c r="C123" s="11" t="inlineStr">
         <is>
-          <t>光镜可判的客观现象（非成败判断）</t>
+          <t>溅射气体与气压</t>
         </is>
       </c>
       <c r="D123" s="11" t="inlineStr">
         <is>
-          <t>下拉+多选</t>
+          <t>下拉+数值</t>
         </is>
       </c>
       <c r="E123" s="11" t="inlineStr">
         <is>
-          <t>无生长/不连续覆盖/厚层区域/可见颗粒沾污/衬底破损/变色/其他</t>
+          <t>Ar / Ar+N₂…</t>
         </is>
       </c>
       <c r="F123" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pa</t>
         </is>
       </c>
       <c r="G123" s="13" t="inlineStr">
@@ -6781,7 +6777,7 @@
       </c>
       <c r="H123" s="11" t="inlineStr">
         <is>
-          <t>不连续覆盖</t>
+          <t>Ar，0.5 Pa</t>
         </is>
       </c>
       <c r="I123" s="11" t="inlineStr">
@@ -6789,32 +6785,32 @@
           <t>复审</t>
         </is>
       </c>
-      <c r="J123" s="15" t="inlineStr">
-        <is>
-          <t>★失败炉次最小痕迹；终态无任何结果→『结果缺失』待办(标准§7/§10)</t>
-        </is>
-      </c>
-      <c r="K123" s="11" t="inlineStr"/>
+      <c r="J123" s="11" t="inlineStr"/>
+      <c r="K123" s="11" t="inlineStr">
+        <is>
+          <t>{"gt":0,"require_value":true}</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="11" t="inlineStr">
         <is>
-          <t>实测产物</t>
+          <t>PVD</t>
         </is>
       </c>
       <c r="B124" s="11" t="inlineStr">
         <is>
-          <t>检出相、多型与堆垛</t>
+          <t>预溅射与挡板时序</t>
         </is>
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>测到的物相/多型/堆垛类型</t>
+          <t>预溅射时长、挡板开合时序</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
         <is>
-          <t>文本</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="E124" s="11" t="inlineStr">
@@ -6824,7 +6820,7 @@
       </c>
       <c r="F124" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>min·s</t>
         </is>
       </c>
       <c r="G124" s="13" t="inlineStr">
@@ -6834,35 +6830,35 @@
       </c>
       <c r="H124" s="11" t="inlineStr">
         <is>
-          <t>2H-MoS₂；AB堆垛</t>
+          <t>预溅 5 min</t>
         </is>
       </c>
       <c r="I124" s="11" t="inlineStr">
         <is>
-          <t>复审/导师</t>
-        </is>
-      </c>
-      <c r="J124" s="15" t="inlineStr">
-        <is>
-          <t>★v3.4导师评审(B76红字)：增记堆垛类型（可判粒度待与俊杰确认，或改下拉）；最小结构化结果</t>
-        </is>
-      </c>
-      <c r="K124" s="11" t="inlineStr"/>
+          <t>复审</t>
+        </is>
+      </c>
+      <c r="J124" s="11" t="inlineStr"/>
+      <c r="K124" s="11" t="inlineStr">
+        <is>
+          <t>{"gt":0}</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="11" t="inlineStr">
         <is>
-          <t>实测产物</t>
+          <t>PVD</t>
         </is>
       </c>
       <c r="B125" s="11" t="inlineStr">
         <is>
-          <t>实测层数</t>
+          <t>沉积速率</t>
         </is>
       </c>
       <c r="C125" s="11" t="inlineStr">
         <is>
-          <t>由表征方法判定的层数</t>
+          <t>速率（QCM 等）</t>
         </is>
       </c>
       <c r="D125" s="11" t="inlineStr">
@@ -6877,7 +6873,7 @@
       </c>
       <c r="F125" s="11" t="inlineStr">
         <is>
-          <t>层</t>
+          <t>nm/s</t>
         </is>
       </c>
       <c r="G125" s="13" t="inlineStr">
@@ -6887,577 +6883,25 @@
       </c>
       <c r="H125" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="I125" s="11" t="inlineStr">
         <is>
-          <t>复审/科学契约审查</t>
-        </is>
-      </c>
-      <c r="J125" s="11" t="inlineStr">
-        <is>
-          <t>历史字段，保留原记录；新表征不录入层数判定，也不将未检出写成层数 0</t>
-        </is>
-      </c>
+          <t>复审</t>
+        </is>
+      </c>
+      <c r="J125" s="11" t="inlineStr"/>
       <c r="K125" s="11" t="inlineStr">
         <is>
-          <t>{"ge":0,"type":"integer"}</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="11" t="inlineStr">
-        <is>
-          <t>实测产物</t>
-        </is>
-      </c>
-      <c r="B126" s="11" t="inlineStr">
-        <is>
-          <t>覆盖率</t>
-        </is>
-      </c>
-      <c r="C126" s="11" t="inlineStr">
-        <is>
-          <t>明确视场或统计区域内材料面积占比</t>
-        </is>
-      </c>
-      <c r="D126" s="11" t="inlineStr">
-        <is>
-          <t>数值</t>
-        </is>
-      </c>
-      <c r="E126" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F126" s="11" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="G126" s="13" t="inlineStr">
-        <is>
-          <t>未发布</t>
-        </is>
-      </c>
-      <c r="H126" s="11" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
-      <c r="I126" s="11" t="inlineStr">
-        <is>
-          <t>复审/科学契约审查</t>
-        </is>
-      </c>
-      <c r="J126" s="11" t="inlineStr">
-        <is>
-          <t>量化口径仍须随表征条件记录</t>
-        </is>
-      </c>
-      <c r="K126" s="11" t="inlineStr">
-        <is>
-          <t>{"ge":0,"le":100}</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="11" t="inlineStr">
-        <is>
-          <t>实测产物</t>
-        </is>
-      </c>
-      <c r="B127" s="11" t="inlineStr">
-        <is>
-          <t>畴尺寸</t>
-        </is>
-      </c>
-      <c r="C127" s="11" t="inlineStr">
-        <is>
-          <t>由指定统计方法得到的代表性畴尺寸</t>
-        </is>
-      </c>
-      <c r="D127" s="11" t="inlineStr">
-        <is>
-          <t>数值</t>
-        </is>
-      </c>
-      <c r="E127" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F127" s="11" t="inlineStr">
-        <is>
-          <t>μm</t>
-        </is>
-      </c>
-      <c r="G127" s="13" t="inlineStr">
-        <is>
-          <t>未发布</t>
-        </is>
-      </c>
-      <c r="H127" s="11" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="I127" s="11" t="inlineStr">
-        <is>
-          <t>复审/科学契约审查</t>
-        </is>
-      </c>
-      <c r="J127" s="11" t="inlineStr"/>
-      <c r="K127" s="11" t="inlineStr">
-        <is>
           <t>{"gt":0}</t>
         </is>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="11" t="inlineStr">
-        <is>
-          <t>实测产物</t>
-        </is>
-      </c>
-      <c r="B128" s="11" t="inlineStr">
-        <is>
-          <t>成核密度</t>
-        </is>
-      </c>
-      <c r="C128" s="11" t="inlineStr">
-        <is>
-          <t>指定统计区域内单位面积成核点数量</t>
-        </is>
-      </c>
-      <c r="D128" s="11" t="inlineStr">
-        <is>
-          <t>数值</t>
-        </is>
-      </c>
-      <c r="E128" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F128" s="11" t="inlineStr">
-        <is>
-          <t>cm⁻²</t>
-        </is>
-      </c>
-      <c r="G128" s="13" t="inlineStr">
-        <is>
-          <t>未发布</t>
-        </is>
-      </c>
-      <c r="H128" s="11" t="inlineStr">
-        <is>
-          <t>10000</t>
-        </is>
-      </c>
-      <c r="I128" s="11" t="inlineStr">
-        <is>
-          <t>复审/科学契约审查</t>
-        </is>
-      </c>
-      <c r="J128" s="11" t="inlineStr"/>
-      <c r="K128" s="11" t="inlineStr">
-        <is>
-          <t>{"ge":0}</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="11" t="inlineStr">
-        <is>
-          <t>实测产物</t>
-        </is>
-      </c>
-      <c r="B129" s="11" t="inlineStr">
-        <is>
-          <t>关键谱学指标</t>
-        </is>
-      </c>
-      <c r="C129" s="11" t="inlineStr">
-        <is>
-          <t>Raman峰位/峰宽/峰面积；PL峰位/峰宽；AFM厚度/粗糙度；SEM覆盖率(视场内材料面积占比,%)/尺寸</t>
-        </is>
-      </c>
-      <c r="D129" s="11" t="inlineStr">
-        <is>
-          <t>结构化指标数组</t>
-        </is>
-      </c>
-      <c r="E129" s="11" t="inlineStr">
-        <is>
-          <t>每条:{metric_code,value,unit}</t>
-        </is>
-      </c>
-      <c r="F129" s="11" t="inlineStr">
-        <is>
-          <t>按指标</t>
-        </is>
-      </c>
-      <c r="G129" s="13" t="inlineStr">
-        <is>
-          <t>未发布</t>
-        </is>
-      </c>
-      <c r="H129" s="11" t="inlineStr">
-        <is>
-          <t>[{"metric_code":"raman_e2g_peak","value":384.2,"unit":"cm-1"}]</t>
-        </is>
-      </c>
-      <c r="I129" s="11" t="inlineStr">
-        <is>
-          <t>复审/导师</t>
-        </is>
-      </c>
-      <c r="J129" s="15" t="inlineStr">
-        <is>
-          <t>★v3.4导师评审(C79红字/K79)：PL补峰宽；『SEM占比』改名『SEM覆盖率』并给定义；随技术选填</t>
-        </is>
-      </c>
-      <c r="K129" s="11" t="inlineStr">
-        <is>
-          <t>{"finite_value":true,"item_required":["metric_code","value","unit"]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="130" ht="20" customHeight="1">
-      <c r="A130" s="10" t="inlineStr">
-        <is>
-          <t>§8 PVD 专用（若合成方法选 PVD 类才启用；延后实现，先占位）</t>
-        </is>
-      </c>
-      <c r="B130" s="8" t="n"/>
-      <c r="C130" s="8" t="n"/>
-      <c r="D130" s="8" t="n"/>
-      <c r="E130" s="8" t="n"/>
-      <c r="F130" s="8" t="n"/>
-      <c r="G130" s="8" t="n"/>
-      <c r="H130" s="8" t="n"/>
-      <c r="I130" s="8" t="n"/>
-      <c r="J130" s="8" t="n"/>
-      <c r="K130" s="8" t="n"/>
-    </row>
-    <row r="131">
-      <c r="A131" s="11" t="inlineStr">
-        <is>
-          <t>PVD</t>
-        </is>
-      </c>
-      <c r="B131" s="11" t="inlineStr">
-        <is>
-          <t>靶材（批次）</t>
-        </is>
-      </c>
-      <c r="C131" s="11" t="inlineStr">
-        <is>
-          <t>靶材化学身份 + 批次</t>
-        </is>
-      </c>
-      <c r="D131" s="11" t="inlineStr">
-        <is>
-          <t>引用</t>
-        </is>
-      </c>
-      <c r="E131" s="11" t="inlineStr">
-        <is>
-          <t>批次库</t>
-        </is>
-      </c>
-      <c r="F131" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G131" s="13" t="inlineStr">
-        <is>
-          <t>未发布</t>
-        </is>
-      </c>
-      <c r="H131" s="11" t="inlineStr">
-        <is>
-          <t>MoS₂ 靶-T01</t>
-        </is>
-      </c>
-      <c r="I131" s="11" t="inlineStr">
-        <is>
-          <t>复审</t>
-        </is>
-      </c>
-      <c r="J131" s="11" t="inlineStr"/>
-      <c r="K131" s="11" t="inlineStr"/>
-    </row>
-    <row r="132">
-      <c r="A132" s="11" t="inlineStr">
-        <is>
-          <t>PVD</t>
-        </is>
-      </c>
-      <c r="B132" s="11" t="inlineStr">
-        <is>
-          <t>靶基距</t>
-        </is>
-      </c>
-      <c r="C132" s="11" t="inlineStr">
-        <is>
-          <t>靶到衬底距离</t>
-        </is>
-      </c>
-      <c r="D132" s="11" t="inlineStr">
-        <is>
-          <t>数值</t>
-        </is>
-      </c>
-      <c r="E132" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F132" s="11" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="G132" s="13" t="inlineStr">
-        <is>
-          <t>未发布</t>
-        </is>
-      </c>
-      <c r="H132" s="11" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="I132" s="11" t="inlineStr">
-        <is>
-          <t>复审</t>
-        </is>
-      </c>
-      <c r="J132" s="11" t="inlineStr"/>
-      <c r="K132" s="11" t="inlineStr">
-        <is>
-          <t>{"gt":0}</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="11" t="inlineStr">
-        <is>
-          <t>PVD</t>
-        </is>
-      </c>
-      <c r="B133" s="11" t="inlineStr">
-        <is>
-          <t>功率与偏压</t>
-        </is>
-      </c>
-      <c r="C133" s="11" t="inlineStr">
-        <is>
-          <t>DC/RF 功率、基底偏压</t>
-        </is>
-      </c>
-      <c r="D133" s="11" t="inlineStr">
-        <is>
-          <t>数值</t>
-        </is>
-      </c>
-      <c r="E133" s="11" t="inlineStr">
-        <is>
-          <t>DC/RF</t>
-        </is>
-      </c>
-      <c r="F133" s="11" t="inlineStr">
-        <is>
-          <t>W·V</t>
-        </is>
-      </c>
-      <c r="G133" s="13" t="inlineStr">
-        <is>
-          <t>未发布</t>
-        </is>
-      </c>
-      <c r="H133" s="11" t="inlineStr">
-        <is>
-          <t>RF 150W；偏压 -50V</t>
-        </is>
-      </c>
-      <c r="I133" s="11" t="inlineStr">
-        <is>
-          <t>复审</t>
-        </is>
-      </c>
-      <c r="J133" s="11" t="inlineStr"/>
-      <c r="K133" s="11" t="inlineStr"/>
-    </row>
-    <row r="134">
-      <c r="A134" s="11" t="inlineStr">
-        <is>
-          <t>PVD</t>
-        </is>
-      </c>
-      <c r="B134" s="11" t="inlineStr">
-        <is>
-          <t>等离子体气氛与工作气压</t>
-        </is>
-      </c>
-      <c r="C134" s="11" t="inlineStr">
-        <is>
-          <t>溅射气体与气压</t>
-        </is>
-      </c>
-      <c r="D134" s="11" t="inlineStr">
-        <is>
-          <t>下拉+数值</t>
-        </is>
-      </c>
-      <c r="E134" s="11" t="inlineStr">
-        <is>
-          <t>Ar / Ar+N₂…</t>
-        </is>
-      </c>
-      <c r="F134" s="11" t="inlineStr">
-        <is>
-          <t>Pa</t>
-        </is>
-      </c>
-      <c r="G134" s="13" t="inlineStr">
-        <is>
-          <t>未发布</t>
-        </is>
-      </c>
-      <c r="H134" s="11" t="inlineStr">
-        <is>
-          <t>Ar，0.5 Pa</t>
-        </is>
-      </c>
-      <c r="I134" s="11" t="inlineStr">
-        <is>
-          <t>复审</t>
-        </is>
-      </c>
-      <c r="J134" s="11" t="inlineStr"/>
-      <c r="K134" s="11" t="inlineStr">
-        <is>
-          <t>{"gt":0,"require_value":true}</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="11" t="inlineStr">
-        <is>
-          <t>PVD</t>
-        </is>
-      </c>
-      <c r="B135" s="11" t="inlineStr">
-        <is>
-          <t>预溅射与挡板时序</t>
-        </is>
-      </c>
-      <c r="C135" s="11" t="inlineStr">
-        <is>
-          <t>预溅射时长、挡板开合时序</t>
-        </is>
-      </c>
-      <c r="D135" s="11" t="inlineStr">
-        <is>
-          <t>数值</t>
-        </is>
-      </c>
-      <c r="E135" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F135" s="11" t="inlineStr">
-        <is>
-          <t>min·s</t>
-        </is>
-      </c>
-      <c r="G135" s="13" t="inlineStr">
-        <is>
-          <t>未发布</t>
-        </is>
-      </c>
-      <c r="H135" s="11" t="inlineStr">
-        <is>
-          <t>预溅 5 min</t>
-        </is>
-      </c>
-      <c r="I135" s="11" t="inlineStr">
-        <is>
-          <t>复审</t>
-        </is>
-      </c>
-      <c r="J135" s="11" t="inlineStr"/>
-      <c r="K135" s="11" t="inlineStr">
-        <is>
-          <t>{"gt":0}</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="11" t="inlineStr">
-        <is>
-          <t>PVD</t>
-        </is>
-      </c>
-      <c r="B136" s="11" t="inlineStr">
-        <is>
-          <t>沉积速率</t>
-        </is>
-      </c>
-      <c r="C136" s="11" t="inlineStr">
-        <is>
-          <t>速率（QCM 等）</t>
-        </is>
-      </c>
-      <c r="D136" s="11" t="inlineStr">
-        <is>
-          <t>数值</t>
-        </is>
-      </c>
-      <c r="E136" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F136" s="11" t="inlineStr">
-        <is>
-          <t>nm/s</t>
-        </is>
-      </c>
-      <c r="G136" s="13" t="inlineStr">
-        <is>
-          <t>未发布</t>
-        </is>
-      </c>
-      <c r="H136" s="11" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="I136" s="11" t="inlineStr">
-        <is>
-          <t>复审</t>
-        </is>
-      </c>
-      <c r="J136" s="11" t="inlineStr"/>
-      <c r="K136" s="11" t="inlineStr">
-        <is>
-          <t>{"gt":0}</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="8">
     <mergeCell ref="A119:K119"/>
     <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A130:K130"/>
     <mergeCell ref="A63:K63"/>
     <mergeCell ref="A47:K47"/>
     <mergeCell ref="A84:K84"/>
@@ -10624,7 +10068,7 @@
       </c>
       <c r="E63" s="11" t="inlineStr">
         <is>
-          <t>OM/Raman/PL/SHG/AFM/SEM/TEM/XRD/其他/低波数Raman</t>
+          <t>OM/Raman/PL/SHG/AFM/SEM/TEM/XRD/其他</t>
         </is>
       </c>
       <c r="F63" s="11" t="inlineStr">

</xml_diff>